<commit_message>
Refresh calibration workbook export
</commit_message>
<xml_diff>
--- a/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_case_review_calibration_6.en.xlsx
+++ b/agent_learning/03_noi_agent/docs/research/dialogue_state_v3_case_review_calibration_6.en.xlsx
@@ -1190,7 +1190,7 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>一个来源大概是已经处理完前面部分后的结果，可我还没说清它对应哪个题目动作。</t>
+          <t>一个来源大概是前面结果，但我还没说清对应哪个动作。</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>一个来源大概是已经处理完前面部分后的结果，可我还没说清它对应哪个题目动作。</t>
+          <t>一个来源大概是前面结果，但我还没说清对应哪个动作。</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>一个来源大概是已经处理完前面部分后的结果，可我还没说清它对应哪个题目动作。</t>
+          <t>一个来源大概是前面结果，但我还没说清对应哪个动作。</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -3000,7 +3000,7 @@
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>一个来源大概是已经处理完前面部分后的结果，可我还没说清它对应哪个题目动作。</t>
+          <t>一个来源大概是前面结果，但我还没说清对应哪个动作。</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">

</xml_diff>